<commit_message>
docs(input_template): regenerate mat strength-view image for the Q:R layout
Point the docs-sheet builder (build_mat) at the master template the docs page
links for download, docs/inputs/input_template.xlsx, rather than the bundled
package copy from default_template_path() — the two lag between a master edit and
the next resource sync, and the rendered image must match the template a reader
downloads. Rebuild sheets_mat.xlsx (phi_b/s_cap now at Q:R, red LEM & FEM
headers) and re-render sheet_mat1.png; the std-dev and seepage views (mat2/mat3)
are unchanged since the move stays inside the strength view. Cells are written by
header name, so the builder is layout-order independent.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0147GB4LGVZuqGHCRMVzZTsR
</commit_message>
<xml_diff>
--- a/docs/usage/sample_sheets/sheets_mat.xlsx
+++ b/docs/usage/sample_sheets/sheets_mat.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/njones/python_projects/xslope/docs/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E9AE3CBE-0B2A-ED44-BB50-AACC6A5490D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{920EFD39-E0D9-5841-8A8C-9199354BBCB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="35040" windowHeight="19900" xr2:uid="{BA54C293-CE08-6E4C-9212-B3317DAA148E}"/>
   </bookViews>
@@ -1421,13 +1421,13 @@
     <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="14" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="14" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1458,7 +1458,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="19">
+  <dxfs count="22">
     <dxf>
       <fill>
         <patternFill>
@@ -1477,6 +1477,27 @@
       <fill>
         <patternFill>
           <bgColor theme="1" tint="0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.499984740745262"/>
         </patternFill>
       </fill>
     </dxf>
@@ -13263,10 +13284,10 @@
       <c r="E2"/>
       <c r="F2"/>
       <c r="G2"/>
-      <c r="N2" s="6" t="s">
+      <c r="L2" s="6" t="s">
         <v>237</v>
       </c>
-      <c r="Q2" s="6" t="s">
+      <c r="O2" s="6" t="s">
         <v>170</v>
       </c>
       <c r="AD2" s="6"/>
@@ -13283,10 +13304,10 @@
       </c>
       <c r="F3"/>
       <c r="G3"/>
-      <c r="Q3" s="1" t="s">
+      <c r="O3" s="1" t="s">
         <v>86</v>
       </c>
-      <c r="R3" t="s">
+      <c r="P3" t="s">
         <v>58</v>
       </c>
       <c r="AD3" s="14"/>
@@ -13306,14 +13327,14 @@
       </c>
       <c r="F4"/>
       <c r="G4"/>
-      <c r="N4" s="42"/>
-      <c r="O4" t="s">
+      <c r="L4" s="42"/>
+      <c r="M4" t="s">
         <v>161</v>
       </c>
-      <c r="Q4" s="1" t="s">
+      <c r="O4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="R4" t="s">
+      <c r="P4" t="s">
         <v>59</v>
       </c>
       <c r="AD4" s="14"/>
@@ -13331,14 +13352,14 @@
       <c r="D5" t="s">
         <v>191</v>
       </c>
-      <c r="N5" s="26"/>
-      <c r="O5" s="9" t="s">
+      <c r="L5" s="26"/>
+      <c r="M5" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="Q5" s="1" t="s">
+      <c r="O5" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="R5" s="9" t="s">
+      <c r="P5" s="9" t="s">
         <v>85</v>
       </c>
       <c r="AD5" s="14"/>
@@ -13356,14 +13377,14 @@
       <c r="D6" s="9" t="s">
         <v>207</v>
       </c>
-      <c r="N6" s="29"/>
-      <c r="O6" s="9" t="s">
+      <c r="L6" s="29"/>
+      <c r="M6" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="Q6" s="1" t="s">
+      <c r="O6" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="R6" t="s">
+      <c r="P6" t="s">
         <v>190</v>
       </c>
       <c r="AE6" s="1"/>
@@ -13459,26 +13480,26 @@
       <c r="K10" s="49" t="s">
         <v>135</v>
       </c>
-      <c r="L10" s="49" t="s">
+      <c r="L10" s="21" t="s">
+        <v>235</v>
+      </c>
+      <c r="M10" s="21" t="s">
+        <v>97</v>
+      </c>
+      <c r="N10" s="43" t="s">
+        <v>211</v>
+      </c>
+      <c r="O10" s="44" t="s">
+        <v>84</v>
+      </c>
+      <c r="P10" s="44" t="s">
+        <v>172</v>
+      </c>
+      <c r="Q10" s="44" t="s">
         <v>238</v>
       </c>
-      <c r="M10" s="49" t="s">
+      <c r="R10" s="44" t="s">
         <v>239</v>
-      </c>
-      <c r="N10" s="21" t="s">
-        <v>235</v>
-      </c>
-      <c r="O10" s="21" t="s">
-        <v>97</v>
-      </c>
-      <c r="P10" s="43" t="s">
-        <v>211</v>
-      </c>
-      <c r="Q10" s="44" t="s">
-        <v>84</v>
-      </c>
-      <c r="R10" s="44" t="s">
-        <v>172</v>
       </c>
       <c r="S10" s="44" t="s">
         <v>173</v>
@@ -13582,26 +13603,26 @@
         <v>20</v>
       </c>
       <c r="L11" s="3">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="M11" s="3">
-        <v>1000</v>
+        <v>30000</v>
       </c>
       <c r="N11" s="3">
-        <v>20</v>
-      </c>
-      <c r="O11" s="3">
-        <v>30000</v>
-      </c>
-      <c r="P11" s="3">
         <v>0.33</v>
       </c>
-      <c r="Q11" s="3" t="inlineStr">
+      <c r="O11" s="3" t="inlineStr">
         <is>
           <t>piezo</t>
         </is>
       </c>
-      <c r="R11" s="3"/>
+      <c r="P11" s="3"/>
+      <c r="Q11" s="3">
+        <v>15</v>
+      </c>
+      <c r="R11" s="3">
+        <v>1000</v>
+      </c>
       <c r="S11" s="3"/>
       <c r="T11" s="3"/>
       <c r="U11" s="3"/>
@@ -13675,22 +13696,22 @@
       </c>
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
-      <c r="L12" s="3"/>
-      <c r="M12" s="3"/>
+      <c r="L12" s="3">
+        <v>0</v>
+      </c>
+      <c r="M12" s="3">
+        <v>8000</v>
+      </c>
       <c r="N12" s="3">
-        <v>0</v>
-      </c>
-      <c r="O12" s="3">
-        <v>8000</v>
-      </c>
-      <c r="P12" s="3">
         <v>0.4</v>
       </c>
-      <c r="Q12" s="3" t="inlineStr">
+      <c r="O12" s="3" t="inlineStr">
         <is>
           <t>piezo</t>
         </is>
       </c>
+      <c r="P12" s="3"/>
+      <c r="Q12" s="3"/>
       <c r="R12" s="3"/>
       <c r="S12" s="3"/>
       <c r="T12" s="3"/>
@@ -13758,19 +13779,19 @@
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
       <c r="L13" s="3"/>
-      <c r="M13" s="3"/>
-      <c r="N13" s="3"/>
-      <c r="O13" s="3">
+      <c r="M13" s="3">
         <v>50000</v>
       </c>
-      <c r="P13" s="3">
+      <c r="N13" s="3">
         <v>0.3</v>
       </c>
-      <c r="Q13" s="3" t="inlineStr">
+      <c r="O13" s="3" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
+      <c r="P13" s="3"/>
+      <c r="Q13" s="3"/>
       <c r="R13" s="3"/>
       <c r="S13" s="3">
         <v>5.5</v>
@@ -13842,19 +13863,19 @@
       <c r="J14" s="3"/>
       <c r="K14" s="3"/>
       <c r="L14" s="3"/>
-      <c r="M14" s="3"/>
-      <c r="N14" s="3"/>
-      <c r="O14" s="3">
+      <c r="M14" s="3">
         <v>500000</v>
       </c>
-      <c r="P14" s="3">
+      <c r="N14" s="3">
         <v>0.25</v>
       </c>
-      <c r="Q14" s="3" t="inlineStr">
+      <c r="O14" s="3" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
+      <c r="P14" s="3"/>
+      <c r="Q14" s="3"/>
       <c r="R14" s="3"/>
       <c r="S14" s="3"/>
       <c r="T14" s="3"/>
@@ -13930,22 +13951,22 @@
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
       <c r="L15" s="3"/>
-      <c r="M15" s="3"/>
-      <c r="N15" s="3"/>
-      <c r="O15" s="3">
+      <c r="M15" s="3">
         <v>40000</v>
       </c>
-      <c r="P15" s="3">
+      <c r="N15" s="3">
         <v>0.3</v>
       </c>
-      <c r="Q15" s="3" t="inlineStr">
+      <c r="O15" s="3" t="inlineStr">
         <is>
           <t>ru</t>
         </is>
       </c>
-      <c r="R15" s="3">
+      <c r="P15" s="3">
         <v>0.15</v>
       </c>
+      <c r="Q15" s="3"/>
+      <c r="R15" s="3"/>
       <c r="S15" s="3"/>
       <c r="T15" s="3"/>
       <c r="U15" s="3"/>
@@ -14010,19 +14031,19 @@
       <c r="J16" s="3"/>
       <c r="K16" s="3"/>
       <c r="L16" s="3"/>
-      <c r="M16" s="3"/>
-      <c r="N16" s="3"/>
-      <c r="O16" s="3">
+      <c r="M16" s="3">
         <v>2000000</v>
       </c>
-      <c r="P16" s="3">
+      <c r="N16" s="3">
         <v>0.22</v>
       </c>
-      <c r="Q16" s="3" t="inlineStr">
+      <c r="O16" s="3" t="inlineStr">
         <is>
           <t>none</t>
         </is>
       </c>
+      <c r="P16" s="3"/>
+      <c r="Q16" s="3"/>
       <c r="R16" s="3"/>
       <c r="S16" s="3"/>
       <c r="T16" s="3"/>
@@ -15119,87 +15140,97 @@
     <mergeCell ref="AG9:AN9"/>
     <mergeCell ref="C9:Z9"/>
   </mergeCells>
-  <conditionalFormatting sqref="L11:M52">
-    <cfRule type="expression" dxfId="5" priority="17">
-      <formula>AND($Q11&lt;&gt;"",$Q11&lt;&gt;"piezo",$Q11&lt;&gt;"seep")</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="F11:K52 AB11:AF52">
-    <cfRule type="expression" dxfId="18" priority="1">
+    <cfRule type="expression" dxfId="21" priority="4">
       <formula>$E11="hb"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="17" priority="2">
+    <cfRule type="expression" dxfId="20" priority="5">
       <formula>$E11="pow"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F11:N52">
-    <cfRule type="expression" dxfId="16" priority="14">
+  <conditionalFormatting sqref="F11:L52">
+    <cfRule type="expression" dxfId="19" priority="17">
       <formula>$E11="elastic"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G11:G52">
-    <cfRule type="expression" dxfId="15" priority="3">
+    <cfRule type="expression" dxfId="18" priority="6">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="H11:I52">
-    <cfRule type="expression" dxfId="14" priority="4">
+    <cfRule type="expression" dxfId="17" priority="7">
       <formula>$E11="mc"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J11:M52">
-    <cfRule type="expression" dxfId="13" priority="5">
+  <conditionalFormatting sqref="J11:K52">
+    <cfRule type="expression" dxfId="16" priority="8">
+      <formula>$E11="cp"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="O11:P52">
+    <cfRule type="expression" dxfId="15" priority="18">
+      <formula>$E11="elastic"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="P11:P52">
+    <cfRule type="expression" dxfId="14" priority="11">
+      <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"ru")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="S11:V52">
+    <cfRule type="expression" dxfId="13" priority="9">
+      <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"pow")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="W11:Z52">
+    <cfRule type="expression" dxfId="12" priority="10">
+      <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"hb")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AB11:AF52">
+    <cfRule type="expression" dxfId="11" priority="19">
+      <formula>$E11="elastic"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AC11:AC52">
+    <cfRule type="expression" dxfId="10" priority="12">
+      <formula>$E11="cp"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AD11:AD52">
+    <cfRule type="expression" dxfId="9" priority="13">
+      <formula>$E11="mc"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AE11:AF52">
+    <cfRule type="expression" dxfId="8" priority="14">
+      <formula>$E11="cp"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AK11:AL52">
+    <cfRule type="expression" dxfId="7" priority="15">
+      <formula>OR($AJ11="vg",$AJ11="gard")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="AM11:AN52">
+    <cfRule type="expression" dxfId="6" priority="16">
+      <formula>$AJ11="lf"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q11:R52">
+    <cfRule type="expression" dxfId="5" priority="2">
+      <formula>$E11="elastic"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="Q11:R52">
+    <cfRule type="expression" dxfId="4" priority="1">
       <formula>$E11="cp"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q11:R52">
-    <cfRule type="expression" dxfId="12" priority="15">
-      <formula>$E11="elastic"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R11:R52">
-    <cfRule type="expression" dxfId="11" priority="8">
-      <formula>AND($Q11&lt;&gt;"",$Q11&lt;&gt;"ru")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S11:V52">
-    <cfRule type="expression" dxfId="10" priority="6">
-      <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"pow")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="W11:Z52">
-    <cfRule type="expression" dxfId="9" priority="7">
-      <formula>AND($E11&lt;&gt;"",$E11&lt;&gt;"hb")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AB11:AF52">
-    <cfRule type="expression" dxfId="8" priority="16">
-      <formula>$E11="elastic"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AC11:AC52">
-    <cfRule type="expression" dxfId="7" priority="9">
-      <formula>$E11="cp"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AD11:AD52">
-    <cfRule type="expression" dxfId="6" priority="10">
-      <formula>$E11="mc"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AE11:AF52">
-    <cfRule type="expression" dxfId="5" priority="11">
-      <formula>$E11="cp"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AK11:AL52">
-    <cfRule type="expression" dxfId="4" priority="12">
-      <formula>OR($AJ11="vg",$AJ11="gard")</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="AM11:AN52">
-    <cfRule type="expression" dxfId="3" priority="13">
-      <formula>$AJ11="lf"</formula>
+    <cfRule type="expression" dxfId="3" priority="3">
+      <formula>AND($O11&lt;&gt;"",$O11&lt;&gt;"piezo",$O11&lt;&gt;"seep")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
@@ -15209,8 +15240,8 @@
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="AJ11:AJ102" xr:uid="{E00A94A9-D864-5843-8FBD-E84775B1C100}">
       <formula1>$AJ$3:$AJ$5</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="Q11:Q52" xr:uid="{D770415C-1ECE-F44B-9D8C-08EF1CF31C8E}">
-      <formula1>$Q$3:$Q$6</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="O11:O52" xr:uid="{D770415C-1ECE-F44B-9D8C-08EF1CF31C8E}">
+      <formula1>$O$3:$O$6</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -15255,74 +15286,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="52" t="s">
+      <c r="A4" s="54" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="52"/>
-      <c r="D4" s="52" t="s">
+      <c r="B4" s="54"/>
+      <c r="D4" s="54" t="s">
         <v>5</v>
       </c>
-      <c r="E4" s="52"/>
-      <c r="G4" s="52" t="s">
+      <c r="E4" s="54"/>
+      <c r="G4" s="54" t="s">
         <v>6</v>
       </c>
-      <c r="H4" s="52"/>
-      <c r="J4" s="52" t="s">
+      <c r="H4" s="54"/>
+      <c r="J4" s="54" t="s">
         <v>7</v>
       </c>
-      <c r="K4" s="52"/>
-      <c r="M4" s="52" t="s">
+      <c r="K4" s="54"/>
+      <c r="M4" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="N4" s="52"/>
-      <c r="P4" s="52" t="s">
+      <c r="N4" s="54"/>
+      <c r="P4" s="54" t="s">
         <v>9</v>
       </c>
-      <c r="Q4" s="52"/>
+      <c r="Q4" s="54"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="52" t="s">
+      <c r="S4" s="54" t="s">
         <v>10</v>
       </c>
-      <c r="T4" s="52"/>
+      <c r="T4" s="54"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="52" t="s">
+      <c r="V4" s="54" t="s">
         <v>11</v>
       </c>
-      <c r="W4" s="52"/>
+      <c r="W4" s="54"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="52" t="s">
+      <c r="Y4" s="54" t="s">
         <v>12</v>
       </c>
-      <c r="Z4" s="52"/>
+      <c r="Z4" s="54"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="52" t="s">
+      <c r="AB4" s="54" t="s">
         <v>13</v>
       </c>
-      <c r="AC4" s="52"/>
-      <c r="AE4" s="52" t="s">
+      <c r="AC4" s="54"/>
+      <c r="AE4" s="54" t="s">
         <v>108</v>
       </c>
-      <c r="AF4" s="52"/>
+      <c r="AF4" s="54"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="52" t="s">
+      <c r="AH4" s="54" t="s">
         <v>109</v>
       </c>
-      <c r="AI4" s="52"/>
+      <c r="AI4" s="54"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="52" t="s">
+      <c r="AK4" s="54" t="s">
         <v>110</v>
       </c>
-      <c r="AL4" s="52"/>
+      <c r="AL4" s="54"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="52" t="s">
+      <c r="AN4" s="54" t="s">
         <v>111</v>
       </c>
-      <c r="AO4" s="52"/>
+      <c r="AO4" s="54"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="52" t="s">
+      <c r="AQ4" s="54" t="s">
         <v>112</v>
       </c>
-      <c r="AR4" s="52"/>
+      <c r="AR4" s="54"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="36" t="s">
@@ -15425,89 +15456,89 @@
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A6" s="53" t="str">
+      <c r="A6" s="52" t="str">
         <f>_xlfn.XLOOKUP(B5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="B6" s="54"/>
-      <c r="D6" s="53" t="str">
+      <c r="B6" s="53"/>
+      <c r="D6" s="52" t="str">
         <f>_xlfn.XLOOKUP(E5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="E6" s="54"/>
-      <c r="G6" s="53" t="str">
+      <c r="E6" s="53"/>
+      <c r="G6" s="52" t="str">
         <f>_xlfn.XLOOKUP(H5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="H6" s="54"/>
-      <c r="J6" s="53" t="str">
+      <c r="H6" s="53"/>
+      <c r="J6" s="52" t="str">
         <f>_xlfn.XLOOKUP(K5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="K6" s="54"/>
-      <c r="M6" s="53" t="str">
+      <c r="K6" s="53"/>
+      <c r="M6" s="52" t="str">
         <f>_xlfn.XLOOKUP(N5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="N6" s="54"/>
-      <c r="P6" s="53" t="str">
+      <c r="N6" s="53"/>
+      <c r="P6" s="52" t="str">
         <f>_xlfn.XLOOKUP(Q5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Q6" s="54"/>
+      <c r="Q6" s="53"/>
       <c r="R6" s="1"/>
-      <c r="S6" s="53" t="str">
+      <c r="S6" s="52" t="str">
         <f>_xlfn.XLOOKUP(T5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="T6" s="54"/>
+      <c r="T6" s="53"/>
       <c r="U6" s="1"/>
-      <c r="V6" s="53" t="str">
+      <c r="V6" s="52" t="str">
         <f>_xlfn.XLOOKUP(W5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="W6" s="54"/>
+      <c r="W6" s="53"/>
       <c r="X6" s="1"/>
-      <c r="Y6" s="53" t="str">
+      <c r="Y6" s="52" t="str">
         <f>_xlfn.XLOOKUP(Z5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="Z6" s="54"/>
+      <c r="Z6" s="53"/>
       <c r="AA6" s="1"/>
-      <c r="AB6" s="53" t="str">
+      <c r="AB6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AC5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AC6" s="54"/>
-      <c r="AE6" s="53" t="str">
+      <c r="AC6" s="53"/>
+      <c r="AE6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AF5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AF6" s="54"/>
+      <c r="AF6" s="53"/>
       <c r="AG6" s="1"/>
-      <c r="AH6" s="53" t="str">
+      <c r="AH6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AI5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AI6" s="54"/>
+      <c r="AI6" s="53"/>
       <c r="AJ6" s="1"/>
-      <c r="AK6" s="53" t="str">
+      <c r="AK6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AL5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AL6" s="54"/>
+      <c r="AL6" s="53"/>
       <c r="AM6" s="1"/>
-      <c r="AN6" s="53" t="str">
+      <c r="AN6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AO5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AO6" s="54"/>
+      <c r="AO6" s="53"/>
       <c r="AP6" s="1"/>
-      <c r="AQ6" s="53" t="str">
+      <c r="AQ6" s="52" t="str">
         <f>_xlfn.XLOOKUP(AR5,mat!$A:$A, mat!$B:$B,"") &amp; ""</f>
         <v/>
       </c>
-      <c r="AR6" s="54"/>
+      <c r="AR6" s="53"/>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A7" s="2" t="s">
@@ -16411,36 +16442,36 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="V4:W4"/>
+    <mergeCell ref="Y4:Z4"/>
+    <mergeCell ref="AB4:AC4"/>
+    <mergeCell ref="AE4:AF4"/>
+    <mergeCell ref="AH4:AI4"/>
+    <mergeCell ref="AK4:AL4"/>
+    <mergeCell ref="AN4:AO4"/>
+    <mergeCell ref="AQ4:AR4"/>
+    <mergeCell ref="A6:B6"/>
+    <mergeCell ref="D6:E6"/>
+    <mergeCell ref="G6:H6"/>
+    <mergeCell ref="J6:K6"/>
+    <mergeCell ref="M6:N6"/>
+    <mergeCell ref="P6:Q6"/>
+    <mergeCell ref="S6:T6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
     <mergeCell ref="AE6:AF6"/>
     <mergeCell ref="AH6:AI6"/>
     <mergeCell ref="AK6:AL6"/>
     <mergeCell ref="AN6:AO6"/>
     <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="P6:Q6"/>
-    <mergeCell ref="S6:T6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="A6:B6"/>
-    <mergeCell ref="D6:E6"/>
-    <mergeCell ref="G6:H6"/>
-    <mergeCell ref="J6:K6"/>
-    <mergeCell ref="M6:N6"/>
-    <mergeCell ref="AE4:AF4"/>
-    <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="AK4:AL4"/>
-    <mergeCell ref="AN4:AO4"/>
-    <mergeCell ref="AQ4:AR4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="S4:T4"/>
-    <mergeCell ref="V4:W4"/>
-    <mergeCell ref="Y4:Z4"/>
-    <mergeCell ref="AB4:AC4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -16478,74 +16509,74 @@
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A4" s="52" t="s">
+      <c r="A4" s="54" t="s">
         <v>137</v>
       </c>
-      <c r="B4" s="52"/>
-      <c r="D4" s="52" t="s">
+      <c r="B4" s="54"/>
+      <c r="D4" s="54" t="s">
         <v>138</v>
       </c>
-      <c r="E4" s="52"/>
-      <c r="G4" s="52" t="s">
+      <c r="E4" s="54"/>
+      <c r="G4" s="54" t="s">
         <v>139</v>
       </c>
-      <c r="H4" s="52"/>
-      <c r="J4" s="52" t="s">
+      <c r="H4" s="54"/>
+      <c r="J4" s="54" t="s">
         <v>140</v>
       </c>
-      <c r="K4" s="52"/>
-      <c r="M4" s="52" t="s">
+      <c r="K4" s="54"/>
+      <c r="M4" s="54" t="s">
         <v>141</v>
       </c>
-      <c r="N4" s="52"/>
-      <c r="P4" s="52" t="s">
+      <c r="N4" s="54"/>
+      <c r="P4" s="54" t="s">
         <v>142</v>
       </c>
-      <c r="Q4" s="52"/>
+      <c r="Q4" s="54"/>
       <c r="R4" s="1"/>
-      <c r="S4" s="52" t="s">
+      <c r="S4" s="54" t="s">
         <v>143</v>
       </c>
-      <c r="T4" s="52"/>
+      <c r="T4" s="54"/>
       <c r="U4" s="1"/>
-      <c r="V4" s="52" t="s">
+      <c r="V4" s="54" t="s">
         <v>144</v>
       </c>
-      <c r="W4" s="52"/>
+      <c r="W4" s="54"/>
       <c r="X4" s="1"/>
-      <c r="Y4" s="52" t="s">
+      <c r="Y4" s="54" t="s">
         <v>145</v>
       </c>
-      <c r="Z4" s="52"/>
+      <c r="Z4" s="54"/>
       <c r="AA4" s="1"/>
-      <c r="AB4" s="52" t="s">
+      <c r="AB4" s="54" t="s">
         <v>146</v>
       </c>
-      <c r="AC4" s="52"/>
-      <c r="AE4" s="52" t="s">
+      <c r="AC4" s="54"/>
+      <c r="AE4" s="54" t="s">
         <v>147</v>
       </c>
-      <c r="AF4" s="52"/>
+      <c r="AF4" s="54"/>
       <c r="AG4" s="1"/>
-      <c r="AH4" s="52" t="s">
+      <c r="AH4" s="54" t="s">
         <v>148</v>
       </c>
-      <c r="AI4" s="52"/>
+      <c r="AI4" s="54"/>
       <c r="AJ4" s="1"/>
-      <c r="AK4" s="52" t="s">
+      <c r="AK4" s="54" t="s">
         <v>149</v>
       </c>
-      <c r="AL4" s="52"/>
+      <c r="AL4" s="54"/>
       <c r="AM4" s="1"/>
-      <c r="AN4" s="52" t="s">
+      <c r="AN4" s="54" t="s">
         <v>150</v>
       </c>
-      <c r="AO4" s="52"/>
+      <c r="AO4" s="54"/>
       <c r="AP4" s="1"/>
-      <c r="AQ4" s="52" t="s">
+      <c r="AQ4" s="54" t="s">
         <v>151</v>
       </c>
-      <c r="AR4" s="52"/>
+      <c r="AR4" s="54"/>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A5" s="38" t="s">
@@ -17634,14 +17665,12 @@
     </row>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="AN6:AO6"/>
-    <mergeCell ref="AQ6:AR6"/>
-    <mergeCell ref="V6:W6"/>
-    <mergeCell ref="Y6:Z6"/>
-    <mergeCell ref="AB6:AC6"/>
-    <mergeCell ref="AE6:AF6"/>
-    <mergeCell ref="AH6:AI6"/>
-    <mergeCell ref="AK6:AL6"/>
+    <mergeCell ref="P4:Q4"/>
+    <mergeCell ref="A4:B4"/>
+    <mergeCell ref="D4:E4"/>
+    <mergeCell ref="G4:H4"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="M4:N4"/>
     <mergeCell ref="AK4:AL4"/>
     <mergeCell ref="AN4:AO4"/>
     <mergeCell ref="AQ4:AR4"/>
@@ -17658,12 +17687,14 @@
     <mergeCell ref="AB4:AC4"/>
     <mergeCell ref="AE4:AF4"/>
     <mergeCell ref="AH4:AI4"/>
-    <mergeCell ref="P4:Q4"/>
-    <mergeCell ref="A4:B4"/>
-    <mergeCell ref="D4:E4"/>
-    <mergeCell ref="G4:H4"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="M4:N4"/>
+    <mergeCell ref="AN6:AO6"/>
+    <mergeCell ref="AQ6:AR6"/>
+    <mergeCell ref="V6:W6"/>
+    <mergeCell ref="Y6:Z6"/>
+    <mergeCell ref="AB6:AC6"/>
+    <mergeCell ref="AE6:AF6"/>
+    <mergeCell ref="AH6:AI6"/>
+    <mergeCell ref="AK6:AL6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>